<commit_message>
Fix #NAME? errors in ESTIMATE Section B: drop leading '=' from result-row labels (openpyxl was writing them as broken formulas); spell out TCC/TFC in Formula/Source column
</commit_message>
<xml_diff>
--- a/1024_G_CEPBKUP_BU26PPE70M_POM26_20260319.xlsx
+++ b/1024_G_CEPBKUP_BU26PPE70M_POM26_20260319.xlsx
@@ -797,9 +797,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="8">
-        <f> Total Contract Cost</f>
-        <v/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Total Contract Cost</t>
+        </is>
       </c>
       <c r="C16" s="6">
         <f>C10*1.10</f>
@@ -828,9 +829,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="8">
-        <f> Total Funded Cost</f>
-        <v/>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Total Funded Cost</t>
+        </is>
       </c>
       <c r="C18" s="6">
         <f>C10*1.10*1.08</f>
@@ -838,7 +840,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>TCC x 1.08</t>
+          <t>Total Contract Cost x 1.08</t>
         </is>
       </c>
     </row>
@@ -859,9 +861,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="8">
-        <f> TOTAL PROJECT COST</f>
-        <v/>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL PROJECT COST</t>
+        </is>
       </c>
       <c r="C20" s="6">
         <f>C10*1.23552</f>
@@ -869,7 +872,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>TFC x 1.04</t>
+          <t>Total Funded Cost x 1.04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild workbooks at PAX's actual rollup rule: DB applied to items (not to TFC); multiplier 1.228 not 1.23552; items subtotal targets calibrated per building so PAX per-step rounding chain produces locked TPC; largest discipline absorbs rounding via plug formula
</commit_message>
<xml_diff>
--- a/1024_G_CEPBKUP_BU26PPE70M_POM26_20260319.xlsx
+++ b/1024_G_CEPBKUP_BU26PPE70M_POM26_20260319.xlsx
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="C9" s="6">
-        <f>C8*PARAMETERS!B37</f>
+        <f>C8*PARAMETERS!B38</f>
         <v/>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -731,14 +731,14 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Equals Locked TPC / 1.23552</t>
+          <t>Calibrated to PAX rollup chain</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>B.  PAX ROLLUP VERIFICATION  (mirrors what PAX prints on the form)</t>
+          <t>B.  PAX ROLLUP VERIFICATION  (mirrors what PAX prints on the form; DB applied to items, not to TFC)</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>From Section A</t>
+          <t>From Section A; pasted into PAX Block 9</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="C15" s="6">
-        <f>C10*0.10</f>
+        <f>ROUND(C10*0.10,0)</f>
         <v/>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -799,16 +799,16 @@
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Total Contract Cost</t>
+          <t>Total Contract Cost (TCC)</t>
         </is>
       </c>
       <c r="C16" s="6">
-        <f>C10*1.10</f>
+        <f>ROUND(C10*1.10,0)</f>
         <v/>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Items Subtotal x 1.10</t>
+          <t>ROUND(items subtotal x 1.10)</t>
         </is>
       </c>
     </row>
@@ -819,28 +819,28 @@
         </is>
       </c>
       <c r="C17" s="6">
-        <f>C10*1.10*0.08</f>
+        <f>ROUND(C16*0.08,0)</f>
         <v/>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>OCONUS FSRM customer-directed</t>
+          <t>OCONUS FSRM customer-directed; ROUND(TCC x 0.08)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Total Funded Cost</t>
+          <t>Total Funded Cost (TFC)</t>
         </is>
       </c>
       <c r="C18" s="6">
-        <f>C10*1.10*1.08</f>
+        <f>ROUND(C16*1.08,0)</f>
         <v/>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Total Contract Cost x 1.08</t>
+          <t>ROUND(TCC x 1.08)</t>
         </is>
       </c>
     </row>
@@ -851,12 +851,12 @@
         </is>
       </c>
       <c r="C19" s="6">
-        <f>C10*1.10*1.08*0.04</f>
+        <f>ROUND(C10*0.04,0)</f>
         <v/>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>UFC 3-730-01 (2024)</t>
+          <t>UFC 3-730-01 (2024); PAX applies DB to items, not to TFC</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
         </is>
       </c>
       <c r="C20" s="6">
-        <f>C10*1.23552</f>
+        <f>C18+C19</f>
         <v/>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Total Funded Cost x 1.04</t>
+          <t>TFC + DB Design  (mirrors PAX Total Request)</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="C21" s="6">
-        <f>ROUND(C20/1000,0)</f>
+        <f>C20</f>
         <v/>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="C24" s="6">
-        <f>C10*0.06</f>
+        <f>ROUND(C10*0.06,0)</f>
         <v/>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -4371,7 +4371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4955,137 +4955,157 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Items Subtotal Target (PAX paste)</t>
-        </is>
-      </c>
-      <c r="B36" s="6">
-        <f>B35/1.23552</f>
-        <v/>
+          <t>Items Subtotal Target ($000)</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>8480</v>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>$</t>
+          <t>$000</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Locked TPC / 1.23552  (1.10 x 1.08 x 1.04)</t>
+          <t>Calibrated so PAX rollup chain (TPC = TFC + DB-on-items) produces Locked TPC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
+          <t>Items Subtotal Target ($)</t>
+        </is>
+      </c>
+      <c r="B37" s="6">
+        <f>B36*1000</f>
+        <v/>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Items Subtotal Target ($000) x 1000</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
           <t>Cost Adjustment Factor</t>
         </is>
       </c>
-      <c r="B37" s="19">
-        <f>B36/B34</f>
-        <v/>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="B38" s="19">
+        <f>B37/B34</f>
+        <v/>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Factor</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>Items Subtotal Target / Pre-Calibration Subtotal; calibrates ROM chain to locked TPC</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Items Subtotal Target / Pre-Calibration Subtotal; calibrates ROM chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>PLANNING RATES</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>JPY/USD Planning Rate</t>
         </is>
       </c>
-      <c r="B40" s="20" t="n">
+      <c r="B41" s="20" t="n">
         <v>150.4415</v>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Rate</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>FY26 budget planning rate; H.10 live rate at PAX submission</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>ACTIVE REFERENCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>MCO 11000.5 (03 Jun 2016)  |  Real Property FSRM Program</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>MCO 11000.12 (08 Sep 2014)  |  Real Property Facilities Manual</t>
+          <t>MCO 11000.5 (03 Jun 2016)  |  Real Property FSRM Program</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Consistency Review Board Guidelines (May 2024, REV #15)  |  DD Form 1391 line-item sequencing</t>
+          <t>MCO 11000.12 (08 Sep 2014)  |  Real Property Facilities Manual</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>UFC 3-701-01 with Change 7 (25 Jul 2025)  |  PUC, ACF, PRV authority</t>
+          <t>Consistency Review Board Guidelines (May 2024, REV #15)  |  DD Form 1391 line-item sequencing</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>UFC 3-730-01 (2024)  |  Design-Build contracting</t>
+          <t>UFC 3-701-01 with Change 7 (25 Jul 2025)  |  PUC, ACF, PRV authority</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>UFS 3-740-05 (02 Feb 2026)  |  Cost estimating ROM levels</t>
+          <t>UFC 3-730-01 (2024)  |  Design-Build contracting</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>JED Cost Estimating Guidance (Combined, Nov 2025)</t>
+          <t>UFS 3-740-05 (02 Feb 2026)  |  Cost estimating ROM levels</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Japan District Design Guide v9 (April 2025)</t>
+          <t>JED Cost Estimating Guidance (Combined, Nov 2025)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Japan District Design Guide v9 (April 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>10 U.S.C. Section 2802  |  DoD 4270.5-M  |  Classification of Work</t>
         </is>
@@ -5095,18 +5115,18 @@
   <mergeCells count="16">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A31:D31"/>
     <mergeCell ref="A50:D50"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A51:D51"/>
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A47:D47"/>
-    <mergeCell ref="A42:D42"/>
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A44:D44"/>
   </mergeCells>
@@ -5166,7 +5186,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"B20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"B20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -5182,7 +5202,7 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"C10",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"C10",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -5198,7 +5218,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"C30",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"C30",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -5214,7 +5234,7 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -5230,7 +5250,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D30",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D30",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -5246,7 +5266,7 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D40",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D40",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -5258,80 +5278,80 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>D50  |  Electrical / Communications</t>
+          <t>E20  |  Furnishings</t>
         </is>
       </c>
       <c r="B10" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"D50",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"E20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>UNIFORMAT II Lv2 D50 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
+          <t>UNIFORMAT II Lv2 E20 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>E20  |  Furnishings</t>
+          <t>F20  |  Selective Demolition</t>
         </is>
       </c>
       <c r="B11" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"E20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"F20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>UNIFORMAT II Lv2 E20 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
+          <t>UNIFORMAT II Lv2 F20 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>F20  |  Selective Demolition</t>
+          <t>G10  |  Site Preparation</t>
         </is>
       </c>
       <c r="B12" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"F20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"G10",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>UNIFORMAT II Lv2 F20 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
+          <t>UNIFORMAT II Lv2 G10 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>G10  |  Site Preparation</t>
+          <t>G20  |  Site Improvements</t>
         </is>
       </c>
       <c r="B13" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"G10",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"G20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B38 / 1000, 0)</f>
         <v/>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>UNIFORMAT II Lv2 G10 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
+          <t>UNIFORMAT II Lv2 G20 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>G20  |  Site Improvements</t>
+          <t>D50  |  Electrical / Communications</t>
         </is>
       </c>
       <c r="B14" s="6">
-        <f>ROUND( SUMIF(SCOPE_DETAIL!H:H,"G20",SCOPE_DETAIL!G:G) * (PARAMETERS!B34/PARAMETERS!B33) * PARAMETERS!B37 / 1000, 0)</f>
+        <f>PARAMETERS!B36-SUM(B4:B13)</f>
         <v/>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>UNIFORMAT II Lv2 G20 rollup; absorbs base-cost adjustments via Cost Adjustment Factor</t>
+          <t>UNIFORMAT II Lv2 D50 rollup; balanced to Items Subtotal Target (absorbs rounding from other rollups)</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5378,7 @@
         </is>
       </c>
       <c r="B17" s="6">
-        <f>B15*0.10</f>
+        <f>ROUND(B15*0.10,0)</f>
         <v/>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -5370,16 +5390,16 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Total Contract Cost</t>
+          <t>Total Contract Cost (TCC)</t>
         </is>
       </c>
       <c r="B18" s="6">
-        <f>B15*1.10</f>
+        <f>ROUND(B15*1.10,0)</f>
         <v/>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Items subtotal x 1.10</t>
+          <t>ROUND(items subtotal x 1.10)</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5410,7 @@
         </is>
       </c>
       <c r="B19" s="6">
-        <f>B15*1.10*0.08</f>
+        <f>ROUND(B18*0.08,0)</f>
         <v/>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -5402,16 +5422,16 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Total Funded Cost</t>
+          <t>Total Funded Cost (TFC)</t>
         </is>
       </c>
       <c r="B20" s="6">
-        <f>B15*1.10*1.08</f>
+        <f>ROUND(B18*1.08,0)</f>
         <v/>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>TCC x 1.08</t>
+          <t>ROUND(TCC x 1.08)</t>
         </is>
       </c>
     </row>
@@ -5422,28 +5442,28 @@
         </is>
       </c>
       <c r="B21" s="6">
-        <f>B15*1.10*1.08*0.04</f>
+        <f>ROUND(B15*0.04,0)</f>
         <v/>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>4% of TFC; UFC 3-730-01 (2024)</t>
+          <t>ROUND(items subtotal x 0.04); PAX applies DB to items, not to TFC</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>TOTAL PROJECT COST</t>
         </is>
       </c>
-      <c r="B22" s="6">
-        <f>B15*1.23552</f>
+      <c r="B22" s="22">
+        <f>B20+B21</f>
         <v/>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>TFC x 1.04 = items subtotal x 1.23552</t>
+          <t>TFC + DB Design  (mirrors PAX Total Request)</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5474,7 @@
         </is>
       </c>
       <c r="B23" s="22">
-        <f>ROUND(B22,0)</f>
+        <f>B22</f>
         <v/>
       </c>
       <c r="C23" s="5" t="inlineStr">

</xml_diff>